<commit_message>
Count an empty Cost or Power as 0 in an uploaded deck
Spell-like cards in a CCG list often have no Power; they now upload as
0-power cards instead of failing the check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TYU7h5Wu8yezZvAgScM8KT
</commit_message>
<xml_diff>
--- a/public/templates/deck-template.xlsx
+++ b/public/templates/deck-template.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Energy needed to play it (a whole number). Required.</t>
+          <t>Energy needed to play it (a whole number). Empty counts as 0.</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Its power at a location (a whole number). Required.</t>
+          <t>Its power at a location (a whole number). Empty counts as 0.</t>
         </is>
       </c>
     </row>

</xml_diff>